<commit_message>
Updated PCA and STRUCTURE
</commit_message>
<xml_diff>
--- a/output/tables/GD/finished tables/GD_temporal_comparisons.xlsx
+++ b/output/tables/GD/finished tables/GD_temporal_comparisons.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30228"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User\Documents\R_WD\revised_bison_popgen\output\tables\GD\finished tables\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\D_RWD\revised_bison_popgen\output\tables\GD\finished tables\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2AA94EE3-40E7-4D84-94CB-363B2D3C4A54}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2D6257EE-5689-491C-B6D5-66117A886529}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-118" yWindow="-118" windowWidth="20343" windowHeight="12934" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="7200" yWindow="210" windowWidth="8550" windowHeight="15270" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -139,6 +139,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="0.000"/>
+  </numFmts>
   <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -214,7 +217,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -237,7 +240,22 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -521,12 +539,13 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:G18"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="16384" width="8.88671875" style="1"/>
+    <col min="1" max="1" width="21.140625" style="1" customWidth="1"/>
+    <col min="2" max="16384" width="8.85546875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="17.05" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:7" ht="16.5" x14ac:dyDescent="0.25">
       <c r="B1" s="7" t="s">
         <v>19</v>
       </c>
@@ -540,7 +559,7 @@
       </c>
       <c r="G1" s="7"/>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" s="4" t="s">
         <v>18</v>
       </c>
@@ -563,375 +582,378 @@
         <v>17</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="B3" s="1">
+        <v>547.5</v>
+      </c>
+      <c r="C3" s="10">
+        <v>0.86553999999999998</v>
+      </c>
+      <c r="D3" s="1">
+        <v>476.5</v>
+      </c>
+      <c r="E3" s="10">
+        <v>0.35721000000000003</v>
+      </c>
+      <c r="F3" s="1">
+        <v>543</v>
+      </c>
+      <c r="G3" s="10">
+        <v>0.82984000000000002</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A4" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="B4" s="1">
+        <v>485</v>
+      </c>
+      <c r="C4" s="10">
+        <v>0.88954999999999995</v>
+      </c>
+      <c r="D4" s="1">
+        <v>533.5</v>
+      </c>
+      <c r="E4" s="10">
+        <v>0.86109999999999998</v>
+      </c>
+      <c r="F4" s="1">
+        <v>424</v>
+      </c>
+      <c r="G4" s="10">
+        <v>0.29383999999999999</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A5" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="B5" s="1">
+        <v>689.5</v>
+      </c>
+      <c r="C5" s="10">
+        <v>0.10467</v>
+      </c>
+      <c r="D5" s="1">
+        <v>619.5</v>
+      </c>
+      <c r="E5" s="10">
+        <v>0.14785000000000001</v>
+      </c>
+      <c r="F5" s="1">
+        <v>810</v>
+      </c>
+      <c r="G5" s="11">
+        <v>8.5000000000000006E-3</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A6" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="B6" s="1">
+        <v>673</v>
+      </c>
+      <c r="C6" s="10">
+        <v>0.25089</v>
+      </c>
+      <c r="D6" s="1">
+        <v>574.5</v>
+      </c>
+      <c r="E6" s="10">
+        <v>0.91571999999999998</v>
+      </c>
+      <c r="F6" s="1">
+        <v>691</v>
+      </c>
+      <c r="G6" s="10">
+        <v>0.18240000000000001</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A7" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="B7" s="1">
+        <v>564</v>
+      </c>
+      <c r="C7" s="10">
+        <v>0.60360000000000003</v>
+      </c>
+      <c r="D7" s="1">
+        <v>505</v>
+      </c>
+      <c r="E7" s="10">
+        <v>0.89224000000000003</v>
+      </c>
+      <c r="F7" s="1">
+        <v>597</v>
+      </c>
+      <c r="G7" s="10">
+        <v>0.37253999999999998</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A8" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="B8" s="1">
+        <v>589</v>
+      </c>
+      <c r="C8" s="10">
+        <v>0.59997999999999996</v>
+      </c>
+      <c r="D8" s="1">
+        <v>542.5</v>
+      </c>
+      <c r="E8" s="10">
+        <v>0.82413000000000003</v>
+      </c>
+      <c r="F8" s="1">
+        <v>676</v>
+      </c>
+      <c r="G8" s="10">
+        <v>0.24048</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A9" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="1">
+      <c r="B9" s="1">
         <v>602.5</v>
       </c>
-      <c r="C3" s="1">
+      <c r="C9" s="10">
         <v>0.50161999999999995</v>
       </c>
-      <c r="D3" s="1">
+      <c r="D9" s="1">
         <v>516.5</v>
       </c>
-      <c r="E3" s="1">
+      <c r="E9" s="10">
         <v>0.79730999999999996</v>
       </c>
-      <c r="F3" s="1">
+      <c r="F9" s="1">
         <v>575</v>
       </c>
-      <c r="G3" s="1">
+      <c r="G9" s="10">
         <v>0.71028999999999998</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A4" s="2" t="s">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A10" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="B10" s="1">
+        <v>576</v>
+      </c>
+      <c r="C10" s="10">
+        <v>0.90314000000000005</v>
+      </c>
+      <c r="D10" s="1">
+        <v>587.5</v>
+      </c>
+      <c r="E10" s="10">
+        <v>0.80767999999999995</v>
+      </c>
+      <c r="F10" s="1">
+        <v>515</v>
+      </c>
+      <c r="G10" s="10">
+        <v>0.61092000000000002</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A11" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="B11" s="1">
+        <v>673</v>
+      </c>
+      <c r="C11" s="10">
+        <v>0.25087999999999999</v>
+      </c>
+      <c r="D11" s="1">
+        <v>619.5</v>
+      </c>
+      <c r="E11" s="10">
+        <v>0.56054000000000004</v>
+      </c>
+      <c r="F11" s="1">
+        <v>715</v>
+      </c>
+      <c r="G11" s="10">
+        <v>0.11179</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A12" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="B12" s="1">
+        <v>611</v>
+      </c>
+      <c r="C12" s="10">
+        <v>0.62265999999999999</v>
+      </c>
+      <c r="D12" s="1">
+        <v>472</v>
+      </c>
+      <c r="E12" s="10">
+        <v>0.33288000000000001</v>
+      </c>
+      <c r="F12" s="1">
+        <v>461</v>
+      </c>
+      <c r="G12" s="10">
+        <v>0.28089999999999998</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A13" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="B13" s="1">
+        <v>652</v>
+      </c>
+      <c r="C13" s="10">
+        <v>0.35446</v>
+      </c>
+      <c r="D13" s="1">
+        <v>546</v>
+      </c>
+      <c r="E13" s="10">
+        <v>0.75185000000000002</v>
+      </c>
+      <c r="F13" s="1">
+        <v>654</v>
+      </c>
+      <c r="G13" s="10">
+        <v>0.34684999999999999</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A14" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="B14" s="1">
+        <v>600.5</v>
+      </c>
+      <c r="C14" s="10">
+        <v>0.70323000000000002</v>
+      </c>
+      <c r="D14" s="1">
+        <v>729</v>
+      </c>
+      <c r="E14" s="10">
+        <v>8.1710000000000005E-2</v>
+      </c>
+      <c r="F14" s="1">
+        <v>579</v>
+      </c>
+      <c r="G14" s="10">
+        <v>0.87919000000000003</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A15" s="8" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="1">
+      <c r="B15" s="9">
         <v>527.5</v>
       </c>
-      <c r="C4" s="1">
+      <c r="C15" s="12">
         <v>0.51422999999999996</v>
       </c>
-      <c r="D4" s="1">
+      <c r="D15" s="9">
         <v>477</v>
       </c>
-      <c r="E4" s="1">
+      <c r="E15" s="12">
         <v>0.83774999999999999</v>
       </c>
-      <c r="F4" s="1" t="s">
+      <c r="F15" s="9" t="s">
         <v>22</v>
       </c>
-      <c r="G4" s="1" t="s">
+      <c r="G15" s="12" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A5" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="B5" s="1">
-        <v>564</v>
-      </c>
-      <c r="C5" s="1">
-        <v>0.60360000000000003</v>
-      </c>
-      <c r="D5" s="1">
-        <v>505</v>
-      </c>
-      <c r="E5" s="1">
-        <v>0.89224000000000003</v>
-      </c>
-      <c r="F5" s="1">
-        <v>597</v>
-      </c>
-      <c r="G5" s="1">
-        <v>0.37253999999999998</v>
-      </c>
-    </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A6" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="B6" s="1">
-        <v>589</v>
-      </c>
-      <c r="C6" s="1">
-        <v>0.59997999999999996</v>
-      </c>
-      <c r="D6" s="1">
-        <v>542.5</v>
-      </c>
-      <c r="E6" s="1">
-        <v>0.82413000000000003</v>
-      </c>
-      <c r="F6" s="1">
-        <v>676</v>
-      </c>
-      <c r="G6" s="1">
-        <v>0.24048</v>
-      </c>
-    </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A7" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="B7" s="1">
-        <v>689.5</v>
-      </c>
-      <c r="C7" s="1">
-        <v>0.10467</v>
-      </c>
-      <c r="D7" s="1">
-        <v>619.5</v>
-      </c>
-      <c r="E7" s="1">
-        <v>0.14785000000000001</v>
-      </c>
-      <c r="F7" s="1">
-        <v>810</v>
-      </c>
-      <c r="G7" s="8">
-        <v>8.5000000000000006E-3</v>
-      </c>
-    </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A8" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="B8" s="1">
-        <v>576</v>
-      </c>
-      <c r="C8" s="1">
-        <v>0.90314000000000005</v>
-      </c>
-      <c r="D8" s="1">
-        <v>587.5</v>
-      </c>
-      <c r="E8" s="1">
-        <v>0.80767999999999995</v>
-      </c>
-      <c r="F8" s="1">
-        <v>515</v>
-      </c>
-      <c r="G8" s="1">
-        <v>0.61092000000000002</v>
-      </c>
-    </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A9" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="B9" s="1">
-        <v>547.5</v>
-      </c>
-      <c r="C9" s="1">
-        <v>0.86553999999999998</v>
-      </c>
-      <c r="D9" s="1">
-        <v>476.5</v>
-      </c>
-      <c r="E9" s="1">
-        <v>0.35721000000000003</v>
-      </c>
-      <c r="F9" s="1">
+    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A16" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="B16" s="1">
+        <v>686.5</v>
+      </c>
+      <c r="C16" s="10">
+        <v>0.19667999999999999</v>
+      </c>
+      <c r="D16" s="1">
+        <v>531.5</v>
+      </c>
+      <c r="E16" s="10">
+        <v>0.73487999999999998</v>
+      </c>
+      <c r="F16" s="1">
+        <v>642</v>
+      </c>
+      <c r="G16" s="10">
+        <v>0.41564000000000001</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A17" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="B17" s="1">
+        <v>601</v>
+      </c>
+      <c r="C17" s="10">
+        <v>0.69930000000000003</v>
+      </c>
+      <c r="D17" s="1">
+        <v>593</v>
+      </c>
+      <c r="E17" s="10">
+        <v>0.39723000000000003</v>
+      </c>
+      <c r="F17" s="1">
         <v>543</v>
       </c>
-      <c r="G9" s="1">
+      <c r="G17" s="10">
         <v>0.82984000000000002</v>
       </c>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A10" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="B10" s="1">
-        <v>485</v>
-      </c>
-      <c r="C10" s="1">
-        <v>0.88954999999999995</v>
-      </c>
-      <c r="D10" s="1">
-        <v>533.5</v>
-      </c>
-      <c r="E10" s="1">
-        <v>0.86109999999999998</v>
-      </c>
-      <c r="F10" s="1">
-        <v>424</v>
-      </c>
-      <c r="G10" s="1">
-        <v>0.29383999999999999</v>
-      </c>
-    </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A11" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="B11" s="1">
-        <v>600.5</v>
-      </c>
-      <c r="C11" s="1">
-        <v>0.70323000000000002</v>
-      </c>
-      <c r="D11" s="1">
-        <v>729</v>
-      </c>
-      <c r="E11" s="1">
-        <v>8.1710000000000005E-2</v>
-      </c>
-      <c r="F11" s="1">
-        <v>579</v>
-      </c>
-      <c r="G11" s="1">
-        <v>0.87919000000000003</v>
-      </c>
-    </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A12" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="B12" s="1">
-        <v>673</v>
-      </c>
-      <c r="C12" s="1">
-        <v>0.25089</v>
-      </c>
-      <c r="D12" s="1">
-        <v>574.5</v>
-      </c>
-      <c r="E12" s="1">
-        <v>0.91571999999999998</v>
-      </c>
-      <c r="F12" s="1">
-        <v>691</v>
-      </c>
-      <c r="G12" s="1">
-        <v>0.18240000000000001</v>
-      </c>
-    </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A13" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="B13" s="1">
-        <v>611</v>
-      </c>
-      <c r="C13" s="1">
-        <v>0.62265999999999999</v>
-      </c>
-      <c r="D13" s="1">
-        <v>472</v>
-      </c>
-      <c r="E13" s="1">
-        <v>0.33288000000000001</v>
-      </c>
-      <c r="F13" s="1">
-        <v>461</v>
-      </c>
-      <c r="G13" s="1">
-        <v>0.28089999999999998</v>
-      </c>
-    </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A14" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="B14" s="1">
-        <v>652</v>
-      </c>
-      <c r="C14" s="1">
-        <v>0.35446</v>
-      </c>
-      <c r="D14" s="1">
-        <v>546</v>
-      </c>
-      <c r="E14" s="1">
-        <v>0.75185000000000002</v>
-      </c>
-      <c r="F14" s="1">
-        <v>654</v>
-      </c>
-      <c r="G14" s="1">
-        <v>0.34684999999999999</v>
-      </c>
-    </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A15" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="B15" s="1">
-        <v>673</v>
-      </c>
-      <c r="C15" s="1">
-        <v>0.25087999999999999</v>
-      </c>
-      <c r="D15" s="1">
-        <v>619.5</v>
-      </c>
-      <c r="E15" s="1">
-        <v>0.56054000000000004</v>
-      </c>
-      <c r="F15" s="1">
-        <v>715</v>
-      </c>
-      <c r="G15" s="1">
-        <v>0.11179</v>
-      </c>
-    </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A16" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="B16" s="1">
-        <v>601</v>
-      </c>
-      <c r="C16" s="1">
-        <v>0.69930000000000003</v>
-      </c>
-      <c r="D16" s="1">
-        <v>593</v>
-      </c>
-      <c r="E16" s="1">
-        <v>0.39723000000000003</v>
-      </c>
-      <c r="F16" s="1">
-        <v>543</v>
-      </c>
-      <c r="G16" s="1">
-        <v>0.82984000000000002</v>
-      </c>
-    </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A17" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="B17" s="1">
-        <v>686.5</v>
-      </c>
-      <c r="C17" s="1">
-        <v>0.19667999999999999</v>
-      </c>
-      <c r="D17" s="1">
-        <v>531.5</v>
-      </c>
-      <c r="E17" s="1">
-        <v>0.73487999999999998</v>
-      </c>
-      <c r="F17" s="1">
-        <v>642</v>
-      </c>
-      <c r="G17" s="1">
-        <v>0.41564000000000001</v>
-      </c>
-    </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:7" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A18" s="3" t="s">
         <v>0</v>
       </c>
       <c r="B18" s="4">
         <v>613.5</v>
       </c>
-      <c r="C18" s="4">
+      <c r="C18" s="13">
         <v>0.42827999999999999</v>
       </c>
       <c r="D18" s="4">
         <v>572</v>
       </c>
-      <c r="E18" s="4">
+      <c r="E18" s="13">
         <v>0.93674000000000002</v>
       </c>
       <c r="F18" s="4">
         <v>685</v>
       </c>
-      <c r="G18" s="4">
+      <c r="G18" s="13">
         <v>0.20427000000000001</v>
       </c>
     </row>
   </sheetData>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A3:G15">
+    <sortCondition ref="A1:A15"/>
+  </sortState>
   <mergeCells count="3">
     <mergeCell ref="B1:C1"/>
     <mergeCell ref="D1:E1"/>

</xml_diff>